<commit_message>
version 0.2 before external feedback
</commit_message>
<xml_diff>
--- a/RSSH-Budget-PF-Dashboard/data/PF outcome and impact mapping.xlsx
+++ b/RSSH-Budget-PF-Dashboard/data/PF outcome and impact mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tommeijer/Git/RSSH-Budget-PF-Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F7F6A3-5379-544B-ACEE-192B3051C0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272557B1-8672-3747-9D60-A7363124CB78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21660" xr2:uid="{3C883CBD-7E49-9C4B-B4C4-89D808B3C730}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="85">
   <si>
     <t>IndicatorCode</t>
   </si>
@@ -288,6 +288,9 @@
   </si>
   <si>
     <t>Removing HRG barriers to TB services</t>
+  </si>
+  <si>
+    <t>TB/HIV</t>
   </si>
 </sst>
 </file>
@@ -1182,7 +1185,7 @@
         <v>51</v>
       </c>
       <c r="B65" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Invoice mngt tool first version and budget PF dashboard ready for testing in streamlit
</commit_message>
<xml_diff>
--- a/RSSH-Budget-PF-Dashboard/data/PF outcome and impact mapping.xlsx
+++ b/RSSH-Budget-PF-Dashboard/data/PF outcome and impact mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tommeijer/Git/RSSH-Budget-PF-Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272557B1-8672-3747-9D60-A7363124CB78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADE3F43-2A1C-1747-80EA-0FFC349D1C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21660" xr2:uid="{3C883CBD-7E49-9C4B-B4C4-89D808B3C730}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="84">
   <si>
     <t>IndicatorCode</t>
   </si>
@@ -288,9 +288,6 @@
   </si>
   <si>
     <t>Removing HRG barriers to TB services</t>
-  </si>
-  <si>
-    <t>TB/HIV</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1182,7 @@
         <v>51</v>
       </c>
       <c r="B65" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>